<commit_message>
Added Unit Testing for Chequing Account and updated its respective Test Plan
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Intermediate Software Development0315\2. Assignments\assignments\assignment_02\instructions\given_files\assignment_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keith\OneDrive\Documents\.RRC\ISD\project\isd-assignment-1\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C65FA7-9822-4725-99C6-8FA3F35E975F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="3555" windowWidth="25185" windowHeight="11415" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -249,6 +249,76 @@
   </si>
   <si>
     <t>Attributes are set to input values (ensure to test for superclass and subclass attributes)</t>
+  </si>
+  <si>
+    <t>Keith Robles</t>
+  </si>
+  <si>
+    <t>Account Number must be numeric, Client Number must be numeric, balance must be a float, date created is valid, overdraft limit must be numeric, and overdraft rate must be numeric</t>
+  </si>
+  <si>
+    <t>account_number = int, client_number = int, balance = float, date_created = date, overdraft_limit = float, and overdraft_rate = float.</t>
+  </si>
+  <si>
+    <t>Inputs are Valid and no Exceptions are Raised</t>
+  </si>
+  <si>
+    <t>overdraft limit is not numeric</t>
+  </si>
+  <si>
+    <t>overdraft rate is not numeric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date created is not a valid type </t>
+  </si>
+  <si>
+    <t>input is not a float or int value</t>
+  </si>
+  <si>
+    <t>overdraft limit is set to -100</t>
+  </si>
+  <si>
+    <t>overdraft rate is set to  0.05</t>
+  </si>
+  <si>
+    <t>input is not a valid date</t>
+  </si>
+  <si>
+    <t>date_created is set to today's date</t>
+  </si>
+  <si>
+    <t>balance is set to a value greater than overdraft limit</t>
+  </si>
+  <si>
+    <t>balance is set to a value less than overdraft limit</t>
+  </si>
+  <si>
+    <t>balance is set to equal to overdraft limit</t>
+  </si>
+  <si>
+    <t>service charge returns value calculated with the formula: BASE_SERVICE_CHARGE + (overdraft limit - balance) * overdraft rate</t>
+  </si>
+  <si>
+    <t>service charge is set to the BASE_SERVICE_CHARGE of 0.5</t>
+  </si>
+  <si>
+    <t>Account Number must be numeric, Client Number must be numeric, balance must be a float, overdraft limit is set a float, and overdraft rate is set to a float.</t>
+  </si>
+  <si>
+    <t>Input is set for the BankAccount class, overdraft limit is a float value, and overdraft rate is a float</t>
+  </si>
+  <si>
+    <t>Outputs like the example: Account Number: 1234567 Balance: $1,559.49
+Overdraft Limit: $-15.00 Overdraft Rate: 5.00% Account Type: Chequing</t>
+  </si>
+  <si>
+    <t>balance value is lower than overdraft limit and overdraft rate is 5 like the example: balance = -600, overdraft limit = -100, overdraft rate = 0.05</t>
+  </si>
+  <si>
+    <t>balance value is higher than overdraft limit and overdraft rate is 5 like the example: balance = 0, overdraft limit = -100, overdraft rate = 0.05</t>
+  </si>
+  <si>
+    <t>balance value is equal overdraft limit and overdraft rate is 5 like the example: balance = -100, overdraft limit = -100, overdraft rate = 0.05</t>
   </si>
 </sst>
 </file>
@@ -1153,18 +1223,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEBCC4-BB44-48CD-B9AB-1E2FD3EE0EEB}">
   <dimension ref="B1:G32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.5703125" customWidth="1"/>
-    <col min="6" max="6" width="28.28515625" customWidth="1"/>
-    <col min="7" max="7" width="48.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="22.26953125" customWidth="1"/>
+    <col min="4" max="4" width="32.7265625" customWidth="1"/>
+    <col min="5" max="5" width="31.54296875" customWidth="1"/>
+    <col min="6" max="6" width="28.26953125" customWidth="1"/>
+    <col min="7" max="7" width="48.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="1.45">
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="2.15">
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -1176,14 +1246,16 @@
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
     </row>
-    <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
+      <c r="C3" s="16" t="s">
+        <v>22</v>
+      </c>
       <c r="D3" s="17"/>
     </row>
-    <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
@@ -1192,10 +1264,10 @@
       </c>
       <c r="D4" s="19"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B6" s="8" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1287,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -1225,11 +1297,17 @@
       <c r="D7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="3">
         <v>2</v>
       </c>
@@ -1239,11 +1317,17 @@
       <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-    </row>
-    <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B9" s="11">
         <v>3</v>
       </c>
@@ -1253,11 +1337,17 @@
       <c r="D9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="12"/>
-    </row>
-    <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="11">
         <v>4</v>
       </c>
@@ -1267,11 +1357,17 @@
       <c r="D10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-    </row>
-    <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="3">
         <v>5</v>
       </c>
@@ -1281,11 +1377,17 @@
       <c r="D11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-    </row>
-    <row r="12" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="11">
         <v>6</v>
       </c>
@@ -1295,11 +1397,17 @@
       <c r="D12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-    </row>
-    <row r="13" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="11">
         <v>7</v>
       </c>
@@ -1309,11 +1417,17 @@
       <c r="D13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B14" s="3">
         <v>8</v>
       </c>
@@ -1323,11 +1437,17 @@
       <c r="D14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B15" s="11">
         <v>9</v>
       </c>
@@ -1337,7 +1457,7 @@
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="11">
         <v>10</v>
       </c>
@@ -1347,7 +1467,7 @@
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="3">
         <v>11</v>
       </c>
@@ -1357,7 +1477,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="11">
         <v>12</v>
       </c>
@@ -1367,7 +1487,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="11">
         <v>13</v>
       </c>
@@ -1377,7 +1497,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B20" s="3">
         <v>14</v>
       </c>
@@ -1387,7 +1507,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="11">
         <v>15</v>
       </c>
@@ -1397,7 +1517,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="11">
         <v>16</v>
       </c>
@@ -1407,7 +1527,7 @@
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B23" s="3">
         <v>17</v>
       </c>
@@ -1417,7 +1537,7 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B24" s="11">
         <v>18</v>
       </c>
@@ -1427,7 +1547,7 @@
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="11">
         <v>19</v>
       </c>
@@ -1437,7 +1557,7 @@
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
     </row>
-    <row r="26" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B26" s="3">
         <v>20</v>
       </c>
@@ -1447,7 +1567,7 @@
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B27" s="11">
         <v>21</v>
       </c>
@@ -1457,7 +1577,7 @@
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="11">
         <v>22</v>
       </c>
@@ -1467,7 +1587,7 @@
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B29" s="3">
         <v>23</v>
       </c>
@@ -1477,7 +1597,7 @@
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B30" s="11">
         <v>24</v>
       </c>
@@ -1487,7 +1607,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="20" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
defined InvestmentAccount and updated their files, alongside Unit Testing for them. Also updated other Unit Tests and their respective Plans
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -2,34 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keith\OneDrive\Documents\.RRC\ISD\project\isd-assignment-1\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keith\Desktop\RRC_Polytech\Winter2025\SoftwareDevFiles_Intermediate\project\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C65FA7-9822-4725-99C6-8FA3F35E975F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D897697-3311-435B-9C28-6E4F82A2AB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="390" yWindow="0" windowWidth="28800" windowHeight="21000" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -161,14 +150,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="1">
     <bk>
       <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
         </ext>
       </extLst>
@@ -308,10 +297,6 @@
     <t>Input is set for the BankAccount class, overdraft limit is a float value, and overdraft rate is a float</t>
   </si>
   <si>
-    <t>Outputs like the example: Account Number: 1234567 Balance: $1,559.49
-Overdraft Limit: $-15.00 Overdraft Rate: 5.00% Account Type: Chequing</t>
-  </si>
-  <si>
     <t>balance value is lower than overdraft limit and overdraft rate is 5 like the example: balance = -600, overdraft limit = -100, overdraft rate = 0.05</t>
   </si>
   <si>
@@ -319,6 +304,10 @@
   </si>
   <si>
     <t>balance value is equal overdraft limit and overdraft rate is 5 like the example: balance = -100, overdraft limit = -100, overdraft rate = 0.05</t>
+  </si>
+  <si>
+    <t>Outputs like the example: "Account Number: 20025 Balance: $0.00 
+Overdraft Limit: $-100.00  Overdraft Rate: 0.05%                 Account Type: Chequing"</t>
   </si>
 </sst>
 </file>
@@ -1223,18 +1212,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEBCC4-BB44-48CD-B9AB-1E2FD3EE0EEB}">
   <dimension ref="B1:G32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.7265625" customWidth="1"/>
-    <col min="3" max="3" width="22.26953125" customWidth="1"/>
-    <col min="4" max="4" width="32.7265625" customWidth="1"/>
-    <col min="5" max="5" width="31.54296875" customWidth="1"/>
-    <col min="6" max="6" width="28.26953125" customWidth="1"/>
-    <col min="7" max="7" width="48.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.5703125" customWidth="1"/>
+    <col min="6" max="6" width="28.28515625" customWidth="1"/>
+    <col min="7" max="7" width="48.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="2.15">
+    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="1.45">
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -1246,7 +1235,7 @@
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
     </row>
-    <row r="3" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
@@ -1255,7 +1244,7 @@
       </c>
       <c r="D3" s="17"/>
     </row>
-    <row r="4" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
@@ -1264,10 +1253,10 @@
       </c>
       <c r="D4" s="19"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8" t="s">
         <v>0</v>
       </c>
@@ -1287,7 +1276,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -1307,7 +1296,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>2</v>
       </c>
@@ -1327,7 +1316,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="11">
         <v>3</v>
       </c>
@@ -1347,7 +1336,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
         <v>4</v>
       </c>
@@ -1367,7 +1356,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>5</v>
       </c>
@@ -1381,13 +1370,13 @@
         <v>34</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11">
         <v>6</v>
       </c>
@@ -1401,13 +1390,13 @@
         <v>35</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G12" s="13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
         <v>7</v>
       </c>
@@ -1421,13 +1410,13 @@
         <v>36</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G13" s="13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>8</v>
       </c>
@@ -1444,10 +1433,10 @@
         <v>40</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="11">
         <v>9</v>
       </c>
@@ -1457,7 +1446,7 @@
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="11">
         <v>10</v>
       </c>
@@ -1467,7 +1456,7 @@
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <v>11</v>
       </c>
@@ -1477,7 +1466,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="11">
         <v>12</v>
       </c>
@@ -1487,7 +1476,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="11">
         <v>13</v>
       </c>
@@ -1497,7 +1486,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
         <v>14</v>
       </c>
@@ -1507,7 +1496,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="11">
         <v>15</v>
       </c>
@@ -1517,7 +1506,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="11">
         <v>16</v>
       </c>
@@ -1527,7 +1516,7 @@
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="3">
         <v>17</v>
       </c>
@@ -1537,7 +1526,7 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11">
         <v>18</v>
       </c>
@@ -1547,7 +1536,7 @@
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="11">
         <v>19</v>
       </c>
@@ -1557,7 +1546,7 @@
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
     </row>
-    <row r="26" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="3">
         <v>20</v>
       </c>
@@ -1567,7 +1556,7 @@
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="11">
         <v>21</v>
       </c>
@@ -1577,7 +1566,7 @@
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="11">
         <v>22</v>
       </c>
@@ -1587,7 +1576,7 @@
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3">
         <v>23</v>
       </c>
@@ -1597,7 +1586,7 @@
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="11">
         <v>24</v>
       </c>
@@ -1607,7 +1596,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="20" t="s">
         <v>6</v>
       </c>

</xml_diff>